<commit_message>
character and scenario card
improved the shared card of character and scenario
</commit_message>
<xml_diff>
--- a/resources/i18n/translations_master.xlsx
+++ b/resources/i18n/translations_master.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="1" r:id="Rbf403f12b4fa4266"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="2" r:id="Rce210d1855b2474f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" r:id="Rff3c0b422936442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="Rbc06c7a9d5474839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="1" r:id="Rf74d86803f6b498a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="2" r:id="R2d542a0dca5449c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" r:id="Rbeb30cfa7bf74f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="R43e0dd6599bb4457"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -886,19 +886,23 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:v>📥 Importer un personnage (JSON)</x:v>
+        <x:v>📥 Importer un personnage partagé</x:v>
       </x:c>
       <x:c r="E17" s="4" t="str">
-        <x:v>📥 Import a character (JSON)</x:v>
+        <x:v>📥 Import shared character</x:v>
       </x:c>
       <x:c r="F17" s="4" t="str">
-        <x:v>📥 Importar un personaje (JSON)</x:v>
+        <x:v>📥 Importar personaje compartido</x:v>
       </x:c>
       <x:c r="G17" s="4" t="str">
-        <x:v>📥 Charakter importieren (JSON)</x:v>
-      </x:c>
-      <x:c r="H17" s="4"/>
-      <x:c r="I17" s="4"/>
+        <x:v>📥 Geteilten Charakter importieren</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>Updated by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I17" s="4" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
       <x:c r="J17" s="4" t="str">
         <x:v>ok</x:v>
       </x:c>
@@ -3244,23 +3248,25 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D97" s="4" t="str">
-        <x:v>Exporter ce personnage (JSON + historique)</x:v>
+        <x:v>Exporter le paquet partageable (fiche + avatar + visages d’humeur)</x:v>
       </x:c>
       <x:c r="E97" s="4" t="str">
-        <x:v>Export this character (JSON + history)</x:v>
+        <x:v>Export share package (profile + avatar + mood faces)</x:v>
       </x:c>
       <x:c r="F97" s="4" t="str">
-        <x:v>Export this character (JSON + history)</x:v>
+        <x:v>Exportar paquete compartible (ficha + avatar + rostros de ánimo)</x:v>
       </x:c>
       <x:c r="G97" s="4" t="str">
-        <x:v>Export this character (JSON + history)</x:v>
+        <x:v>Teilbares Paket exportieren (Profil + Avatar + Stimmungsbilder)</x:v>
       </x:c>
       <x:c r="H97" s="4" t="str">
-        <x:v>English fallback pending localized review</x:v>
-      </x:c>
-      <x:c r="I97" s="4"/>
+        <x:v>Updated by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I97" s="4" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
       <x:c r="J97" s="4" t="str">
-        <x:v>fallback_en</x:v>
+        <x:v>ok</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -30942,19 +30948,19 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D985" t="str">
-        <x:v>40.0.4</x:v>
+        <x:v>40.0.8</x:v>
       </x:c>
       <x:c r="E985" t="str">
-        <x:v>40.0.4</x:v>
+        <x:v>40.0.8</x:v>
       </x:c>
       <x:c r="F985" t="str">
-        <x:v>40.0.4</x:v>
+        <x:v>40.0.8</x:v>
       </x:c>
       <x:c r="G985" t="str">
-        <x:v>40.0.4</x:v>
+        <x:v>40.0.8</x:v>
       </x:c>
       <x:c r="H985" t="str">
-        <x:v>Updated by v40.0.4 GitHub licence and copyright patch</x:v>
+        <x:v>Updated by v40.0.8 public share packages</x:v>
       </x:c>
       <x:c r="I985" t="str">
         <x:v>resources/i18n/locales/*.json</x:v>
@@ -31280,6 +31286,358 @@
         <x:v>resources/i18n/locales/*.json</x:v>
       </x:c>
       <x:c r="J995" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="996">
+      <x:c r="A996" t="str">
+        <x:v>scenario.import_btn</x:v>
+      </x:c>
+      <x:c r="B996" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C996" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D996" t="str">
+        <x:v>📥 Importer un scénario partagé</x:v>
+      </x:c>
+      <x:c r="E996" t="str">
+        <x:v>📥 Import shared scenario</x:v>
+      </x:c>
+      <x:c r="F996" t="str">
+        <x:v>📥 Importar escenario compartido</x:v>
+      </x:c>
+      <x:c r="G996" t="str">
+        <x:v>📥 Geteiltes Szenario importieren</x:v>
+      </x:c>
+      <x:c r="H996" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I996" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J996" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="997">
+      <x:c r="A997" t="str">
+        <x:v>scenario.share_hint</x:v>
+      </x:c>
+      <x:c r="B997" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C997" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D997" t="str">
+        <x:v>Les paquets de scénario partagés contiennent uniquement les données narratives.</x:v>
+      </x:c>
+      <x:c r="E997" t="str">
+        <x:v>Shared scenario packages contain narrative data only.</x:v>
+      </x:c>
+      <x:c r="F997" t="str">
+        <x:v>Los paquetes de escenario compartidos solo contienen datos narrativos.</x:v>
+      </x:c>
+      <x:c r="G997" t="str">
+        <x:v>Geteilte Szenariopakete enthalten ausschließlich narrative Daten.</x:v>
+      </x:c>
+      <x:c r="H997" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I997" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J997" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="998">
+      <x:c r="A998" t="str">
+        <x:v>scenario.export_btn</x:v>
+      </x:c>
+      <x:c r="B998" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C998" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D998" t="str">
+        <x:v>📤 Partager</x:v>
+      </x:c>
+      <x:c r="E998" t="str">
+        <x:v>📤 Share</x:v>
+      </x:c>
+      <x:c r="F998" t="str">
+        <x:v>📤 Compartir</x:v>
+      </x:c>
+      <x:c r="G998" t="str">
+        <x:v>📤 Teilen</x:v>
+      </x:c>
+      <x:c r="H998" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I998" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J998" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="999">
+      <x:c r="A999" t="str">
+        <x:v>scenario.edit_btn</x:v>
+      </x:c>
+      <x:c r="B999" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C999" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D999" t="str">
+        <x:v>✏️ Modifier</x:v>
+      </x:c>
+      <x:c r="E999" t="str">
+        <x:v>✏️ Edit</x:v>
+      </x:c>
+      <x:c r="F999" t="str">
+        <x:v>✏️ Editar</x:v>
+      </x:c>
+      <x:c r="G999" t="str">
+        <x:v>✏️ Bearbeiten</x:v>
+      </x:c>
+      <x:c r="H999" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I999" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J999" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1000">
+      <x:c r="A1000" t="str">
+        <x:v>scenario.delete_confirm</x:v>
+      </x:c>
+      <x:c r="B1000" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C1000" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1000" t="str">
+        <x:v>Supprimer ce scénario ?</x:v>
+      </x:c>
+      <x:c r="E1000" t="str">
+        <x:v>Delete this scenario?</x:v>
+      </x:c>
+      <x:c r="F1000" t="str">
+        <x:v>¿Eliminar este escenario?</x:v>
+      </x:c>
+      <x:c r="G1000" t="str">
+        <x:v>Dieses Szenario löschen?</x:v>
+      </x:c>
+      <x:c r="H1000" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I1000" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1000" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1001">
+      <x:c r="A1001" t="str">
+        <x:v>scenario.apply_title</x:v>
+      </x:c>
+      <x:c r="B1001" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C1001" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1001" t="str">
+        <x:v>Appliquer à la conversation active</x:v>
+      </x:c>
+      <x:c r="E1001" t="str">
+        <x:v>Apply to active conversation</x:v>
+      </x:c>
+      <x:c r="F1001" t="str">
+        <x:v>Aplicar a la conversación activa</x:v>
+      </x:c>
+      <x:c r="G1001" t="str">
+        <x:v>Auf die aktive Unterhaltung anwenden</x:v>
+      </x:c>
+      <x:c r="H1001" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I1001" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1001" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1002">
+      <x:c r="A1002" t="str">
+        <x:v>scenario.apply_btn</x:v>
+      </x:c>
+      <x:c r="B1002" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C1002" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1002" t="str">
+        <x:v>▶ Appliquer</x:v>
+      </x:c>
+      <x:c r="E1002" t="str">
+        <x:v>▶ Apply</x:v>
+      </x:c>
+      <x:c r="F1002" t="str">
+        <x:v>▶ Aplicar</x:v>
+      </x:c>
+      <x:c r="G1002" t="str">
+        <x:v>▶ Anwenden</x:v>
+      </x:c>
+      <x:c r="H1002" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I1002" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1002" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1003">
+      <x:c r="A1003" t="str">
+        <x:v>scenario.import_success</x:v>
+      </x:c>
+      <x:c r="B1003" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C1003" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1003" t="str">
+        <x:v>Scénario « {title} » importé !</x:v>
+      </x:c>
+      <x:c r="E1003" t="str">
+        <x:v>Scenario “{title}” imported!</x:v>
+      </x:c>
+      <x:c r="F1003" t="str">
+        <x:v>¡Escenario «{title}» importado!</x:v>
+      </x:c>
+      <x:c r="G1003" t="str">
+        <x:v>Szenario „{title}“ importiert!</x:v>
+      </x:c>
+      <x:c r="H1003" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I1003" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1003" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1004">
+      <x:c r="A1004" t="str">
+        <x:v>scenario.import_failed</x:v>
+      </x:c>
+      <x:c r="B1004" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="C1004" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1004" t="str">
+        <x:v>Échec de l’import du scénario : {error}</x:v>
+      </x:c>
+      <x:c r="E1004" t="str">
+        <x:v>Scenario import failed: {error}</x:v>
+      </x:c>
+      <x:c r="F1004" t="str">
+        <x:v>Error al importar el escenario: {error}</x:v>
+      </x:c>
+      <x:c r="G1004" t="str">
+        <x:v>Szenarioimport fehlgeschlagen: {error}</x:v>
+      </x:c>
+      <x:c r="H1004" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I1004" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1004" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1005">
+      <x:c r="A1005" t="str">
+        <x:v>char.share_hint</x:v>
+      </x:c>
+      <x:c r="B1005" t="str">
+        <x:v>char</x:v>
+      </x:c>
+      <x:c r="C1005" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1005" t="str">
+        <x:v>Paquet public : les conversations, mémoires personnelles, voix et réglages ne sont jamais inclus.</x:v>
+      </x:c>
+      <x:c r="E1005" t="str">
+        <x:v>Public package: conversations, personal memories, voice and settings are never included.</x:v>
+      </x:c>
+      <x:c r="F1005" t="str">
+        <x:v>Paquete público: nunca se incluyen conversaciones, recuerdos personales, voz ni ajustes.</x:v>
+      </x:c>
+      <x:c r="G1005" t="str">
+        <x:v>Öffentliches Paket: Unterhaltungen, persönliche Erinnerungen, Stimme und Einstellungen werden niemals eingeschlossen.</x:v>
+      </x:c>
+      <x:c r="H1005" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I1005" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1005" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1006">
+      <x:c r="A1006" t="str">
+        <x:v>char.share_btn</x:v>
+      </x:c>
+      <x:c r="B1006" t="str">
+        <x:v>char</x:v>
+      </x:c>
+      <x:c r="C1006" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1006" t="str">
+        <x:v>📤 Partager</x:v>
+      </x:c>
+      <x:c r="E1006" t="str">
+        <x:v>📤 Share</x:v>
+      </x:c>
+      <x:c r="F1006" t="str">
+        <x:v>📤 Compartir</x:v>
+      </x:c>
+      <x:c r="G1006" t="str">
+        <x:v>📤 Teilen</x:v>
+      </x:c>
+      <x:c r="H1006" t="str">
+        <x:v>Added by v40.0.8 public share packages</x:v>
+      </x:c>
+      <x:c r="I1006" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1006" t="str">
         <x:v>ok</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
run pod and serverless addition
</commit_message>
<xml_diff>
--- a/resources/i18n/translations_master.xlsx
+++ b/resources/i18n/translations_master.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="1" r:id="R1f966a4abed0466e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="2" r:id="R4994c2dd9be74e95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" r:id="Rc372d3b3e4ba421a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="Rda33240f16e94c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="1" r:id="Rd1aa8191aa4c4ab3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="2" r:id="Ra73f54a19ce94835"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" r:id="R884fac50eb7f4a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="R81dc7d16a4f14097"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -802,19 +802,23 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D14" s="3" t="str">
-        <x:v>100 % local — LLM + ComfyUI</x:v>
+        <x:v>Local d’abord — moteurs locaux ou services personnels</x:v>
       </x:c>
       <x:c r="E14" s="3" t="str">
-        <x:v>100% local — LLM + ComfyUI</x:v>
+        <x:v>Local-first — local or user-owned AI engines</x:v>
       </x:c>
       <x:c r="F14" s="3" t="str">
-        <x:v>100% local — LLM + ComfyUI</x:v>
+        <x:v>Local primero — motores locales o servicios propios</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
-        <x:v>100% lokal — LLM + ComfyUI</x:v>
-      </x:c>
-      <x:c r="H14" s="3"/>
-      <x:c r="I14" s="3"/>
+        <x:v>Local-first — lokale oder eigene KI-Dienste</x:v>
+      </x:c>
+      <x:c r="H14" s="3" t="str">
+        <x:v>Updated by v40.1.0 remote providers</x:v>
+      </x:c>
+      <x:c r="I14" s="3" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
       <x:c r="J14" s="3" t="str">
         <x:v>ok</x:v>
       </x:c>
@@ -9576,23 +9580,25 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D309" s="4" t="str">
-        <x:v>Un seul programme charge ton LLM et ton modèle image. Tout reste sur ta machine.</x:v>
+        <x:v>Choisis des moteurs locaux ou connecte tes propres services. Les données du compagnon restent locales ; seuls les appels envoyés à un fournisseur distant le quittent.</x:v>
       </x:c>
       <x:c r="E309" s="4" t="str">
-        <x:v>One program loads your LLM and image model. Everything stays on your machine.</x:v>
+        <x:v>Choose local engines or connect services you own. Companion data stays local; remote providers receive only requests sent to them.</x:v>
       </x:c>
       <x:c r="F309" s="4" t="str">
-        <x:v>One program loads your LLM and image model. Everything stays on your machine.</x:v>
+        <x:v>Elige motores locales o conecta tus propios servicios. Los datos del compañero permanecen locales; solo salen las solicitudes enviadas a un proveedor remoto.</x:v>
       </x:c>
       <x:c r="G309" s="4" t="str">
-        <x:v>One program loads your LLM and image model. Everything stays on your machine.</x:v>
+        <x:v>Wähle lokale Engines oder verbinde eigene Dienste. Begleiterdaten bleiben lokal; nur ausdrücklich gesendete Remote-Anfragen verlassen den PC.</x:v>
       </x:c>
       <x:c r="H309" s="4" t="str">
-        <x:v>English fallback pending localized review</x:v>
-      </x:c>
-      <x:c r="I309" s="4"/>
+        <x:v>Updated by v40.1.0 remote providers</x:v>
+      </x:c>
+      <x:c r="I309" s="4" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
       <x:c r="J309" s="4" t="str">
-        <x:v>fallback_en</x:v>
+        <x:v>ok</x:v>
       </x:c>
     </x:row>
     <x:row r="310">
@@ -10372,16 +10378,16 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D336" s="4" t="str">
-        <x:v>Cette valeur doit rester égale ou inférieure au contexte réellement configuré pour le modèle dans LM Studio.</x:v>
+        <x:v>Cette valeur doit rester égale ou inférieure au contexte réellement configuré pour le modèle chez le fournisseur sélectionné.</x:v>
       </x:c>
       <x:c r="E336" s="4" t="str">
-        <x:v>This value must be equal to or less than the context actually configured for the model in LM Studio.</x:v>
+        <x:v>This value must be equal to or lower than the context actually configured for the model on the selected provider.</x:v>
       </x:c>
       <x:c r="F336" s="4" t="str">
-        <x:v>This value must be equal to or less than the context actually configured for the model in LM Studio.</x:v>
+        <x:v>Este valor debe ser igual o inferior al contexto configurado realmente para el modelo en el proveedor seleccionado.</x:v>
       </x:c>
       <x:c r="G336" s="4" t="str">
-        <x:v>This value must be equal to or less than the context actually configured for the model in LM Studio.</x:v>
+        <x:v>Dieser Wert muss kleiner oder gleich dem tatsächlich beim ausgewählten Anbieter konfigurierten Modellkontext sein.</x:v>
       </x:c>
       <x:c r="H336" s="4" t="str">
         <x:v>English fallback pending localized review</x:v>
@@ -10489,26 +10495,28 @@
         <x:v>settings</x:v>
       </x:c>
       <x:c r="C340" s="4" t="str">
-        <x:v>text</x:v>
+        <x:v>html</x:v>
       </x:c>
       <x:c r="D340" s="4" t="str">
-        <x:v>Astuce qualité : un modèle de &lt;b&gt;roleplay&lt;/b&gt; (souvent non censuré) est mauvais pour produire du JSON propre et des prompts d'image structurés.</x:v>
+        <x:v>Astuce qualité : un modèle de &lt;b&gt;roleplay&lt;/b&gt; (souvent non censuré) est mauvais pour produire du JSON propre et des prompts d’image structurés.</x:v>
       </x:c>
       <x:c r="E340" s="4" t="str">
         <x:v>Quality tip: a &lt;b&gt;roleplay&lt;/b&gt; model (often uncensored) is poor at producing clean JSON and structured image prompts.</x:v>
       </x:c>
       <x:c r="F340" s="4" t="str">
-        <x:v>Quality tip: a &lt;b&gt;roleplay&lt;/b&gt; model (often uncensored) is poor at producing clean JSON and structured image prompts.</x:v>
+        <x:v>Consejo de calidad: un modelo de &lt;b&gt;roleplay&lt;/b&gt; (a menudo sin censura) suele producir peor JSON limpio y prompts de imagen estructurados.</x:v>
       </x:c>
       <x:c r="G340" s="4" t="str">
-        <x:v>Quality tip: a &lt;b&gt;roleplay&lt;/b&gt; model (often uncensored) is poor at producing clean JSON and structured image prompts.</x:v>
+        <x:v>Qualitätstipp: Ein &lt;b&gt;Roleplay&lt;/b&gt;-Modell (oft unzensiert) eignet sich meist schlecht für sauberes JSON und strukturierte Bild-Prompts.</x:v>
       </x:c>
       <x:c r="H340" s="4" t="str">
-        <x:v>English fallback pending localized review</x:v>
-      </x:c>
-      <x:c r="I340" s="4"/>
+        <x:v>Corrected ES/DE and retained by v40.1.0</x:v>
+      </x:c>
+      <x:c r="I340" s="4" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
       <x:c r="J340" s="4" t="str">
-        <x:v>fallback_en</x:v>
+        <x:v>ok</x:v>
       </x:c>
     </x:row>
     <x:row r="341">
@@ -11044,19 +11052,19 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D358" s="4" t="str">
-        <x:v>Connexion ComfyUI tiers</x:v>
+        <x:v>Fournisseur de génération d’images</x:v>
       </x:c>
       <x:c r="E358" s="4" t="str">
-        <x:v>External ComfyUI connection</x:v>
+        <x:v>Image generation provider</x:v>
       </x:c>
       <x:c r="F358" s="4" t="str">
-        <x:v>Conexión con ComfyUI externo</x:v>
+        <x:v>Proveedor de generación de imágenes</x:v>
       </x:c>
       <x:c r="G358" s="4" t="str">
-        <x:v>Verbindung zu externem ComfyUI</x:v>
+        <x:v>Anbieter für Bildgenerierung</x:v>
       </x:c>
       <x:c r="H358" s="4" t="str">
-        <x:v>v40.0.7 external ComfyUI only</x:v>
+        <x:v>Updated by v40.1.0 remote image providers</x:v>
       </x:c>
       <x:c r="I358" s="4" t="str">
         <x:v>resources/i18n/locales/*.json</x:v>
@@ -11076,19 +11084,19 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D359" s="4" t="str">
-        <x:v>AmiorAI se connecte uniquement à une installation ComfyUI tierce déjà démarrée. Il n’installe, ne lance, ne redémarre et n’arrête jamais ComfyUI. Les modèles et workflows se choisissent dans &lt;strong&gt;Studio Image&lt;/strong&gt;.</x:v>
+        <x:v>Choisis un moteur d’image local ou distant qui t’appartient. AmiorAI ne vend pas de calcul et ne gère pas la facturation du fournisseur.</x:v>
       </x:c>
       <x:c r="E359" s="4" t="str">
-        <x:v>AmiorAI only connects to an already running third-party ComfyUI installation. It never installs, launches, restarts or stops ComfyUI. Image models and workflows are selected in &lt;strong&gt;Image Studio&lt;/strong&gt;.</x:v>
+        <x:v>Choose a local or user-owned remote image engine. AmiorAI does not sell compute and does not manage provider billing.</x:v>
       </x:c>
       <x:c r="F359" s="4" t="str">
-        <x:v>AmiorAI solo se conecta a una instalación de ComfyUI de terceros que ya esté en ejecución. Nunca instala, inicia, reinicia ni detiene ComfyUI. Los modelos y flujos de trabajo se eligen en &lt;strong&gt;Estudio de imágenes&lt;/strong&gt;.</x:v>
+        <x:v>Elige un motor de imágenes local o remoto de tu propiedad. AmiorAI no vende cómputo ni gestiona la facturación.</x:v>
       </x:c>
       <x:c r="G359" s="4" t="str">
-        <x:v>AmiorAI verbindet sich nur mit einer bereits laufenden ComfyUI-Installation eines Drittanbieters. ComfyUI wird niemals von AmiorAI installiert, gestartet, neu gestartet oder beendet. Modelle und Workflows werden in &lt;strong&gt;Image Studio&lt;/strong&gt; ausgewählt.</x:v>
+        <x:v>Wähle eine lokale oder eigene entfernte Bild-Engine. AmiorAI verkauft keine Rechenleistung und verwaltet keine Anbieterabrechnung.</x:v>
       </x:c>
       <x:c r="H359" s="4" t="str">
-        <x:v>v40.0.7 external ComfyUI only</x:v>
+        <x:v>Updated by v40.1.0 remote image providers</x:v>
       </x:c>
       <x:c r="I359" s="4" t="str">
         <x:v>resources/i18n/locales/*.json</x:v>
@@ -28484,19 +28492,19 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="D908" s="28" t="str">
-        <x:v>Le modèle utilitaire utilise le même serveur LM Studio et la même clé API.</x:v>
+        <x:v>Le modèle utilitaire utilise le même fournisseur et les mêmes identifiants que le modèle conversationnel.</x:v>
       </x:c>
       <x:c r="E908" s="28" t="str">
-        <x:v>The utility model uses the same LM Studio server and API key.</x:v>
+        <x:v>The utility model uses the same selected provider and credentials as the conversation model.</x:v>
       </x:c>
       <x:c r="F908" s="28" t="str">
-        <x:v>El modelo utilitario usa el mismo servidor LM Studio y la misma clave API.</x:v>
+        <x:v>El modelo utilitario usa el mismo proveedor y las mismas credenciales que el modelo de conversación.</x:v>
       </x:c>
       <x:c r="G908" s="28" t="str">
-        <x:v>Das Hilfsmodell verwendet denselben LM-Studio-Server und API-Schlüssel.</x:v>
+        <x:v>Das Hilfsmodell verwendet denselben ausgewählten Anbieter und dieselben Zugangsdaten wie das Konversationsmodell.</x:v>
       </x:c>
       <x:c r="H908" s="28" t="str">
-        <x:v>Added by v39.1.0 non-destructive merge</x:v>
+        <x:v>Updated by v40.1.0 provider abstraction</x:v>
       </x:c>
       <x:c r="I908" s="28" t="str">
         <x:v>resources/i18n/locales/*.json</x:v>
@@ -31926,6 +31934,1990 @@
         <x:v>resources/i18n/locales/*.json</x:v>
       </x:c>
       <x:c r="J1015" s="28" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1016">
+      <x:c r="A1016" t="str">
+        <x:v>settings.providers_privacy_hint</x:v>
+      </x:c>
+      <x:c r="B1016" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1016" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1016" t="str">
+        <x:v>Le mode local garde les prompts sur ce PC. Les modes distants envoient uniquement les données nécessaires à la tâche au fournisseur configuré par l’utilisateur.</x:v>
+      </x:c>
+      <x:c r="E1016" t="str">
+        <x:v>Local mode keeps prompts on this PC. Remote modes send only the data required for the selected task to the provider configured by the user.</x:v>
+      </x:c>
+      <x:c r="F1016" t="str">
+        <x:v>El modo local conserva los prompts en este PC. Los modos remotos envían únicamente los datos necesarios al proveedor configurado por el usuario.</x:v>
+      </x:c>
+      <x:c r="G1016" t="str">
+        <x:v>Im lokalen Modus bleiben Prompts auf diesem PC. Remote-Modi senden nur die für die Aufgabe nötigen Daten an den vom Benutzer konfigurierten Anbieter.</x:v>
+      </x:c>
+      <x:c r="H1016" t="str">
+        <x:v>Added by v40.1.0 remote providers</x:v>
+      </x:c>
+      <x:c r="I1016" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1016" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1017">
+      <x:c r="A1017" t="str">
+        <x:v>settings.llm_provider_label</x:v>
+      </x:c>
+      <x:c r="B1017" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1017" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1017" t="str">
+        <x:v>Fournisseur de conversation</x:v>
+      </x:c>
+      <x:c r="E1017" t="str">
+        <x:v>Conversation provider</x:v>
+      </x:c>
+      <x:c r="F1017" t="str">
+        <x:v>Proveedor de conversación</x:v>
+      </x:c>
+      <x:c r="G1017" t="str">
+        <x:v>Konversationsanbieter</x:v>
+      </x:c>
+      <x:c r="H1017" t="str">
+        <x:v>Added by v40.1.0 remote LLM providers</x:v>
+      </x:c>
+      <x:c r="I1017" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1017" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1018">
+      <x:c r="A1018" t="str">
+        <x:v>settings.image_provider_hint</x:v>
+      </x:c>
+      <x:c r="B1018" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1018" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1018" t="str">
+        <x:v>Choisis ComfyUI local, un serveur ComfyUI distant, Runpod Serverless ou ton propre Pod Runpod.</x:v>
+      </x:c>
+      <x:c r="E1018" t="str">
+        <x:v>Choose local ComfyUI, a remote ComfyUI-compatible server, Runpod Serverless, or a user-owned Runpod Pod.</x:v>
+      </x:c>
+      <x:c r="F1018" t="str">
+        <x:v>Elige ComfyUI local, un servidor ComfyUI remoto, Runpod Serverless o tu propio Pod de Runpod.</x:v>
+      </x:c>
+      <x:c r="G1018" t="str">
+        <x:v>Wähle lokales ComfyUI, einen entfernten ComfyUI-Server, Runpod Serverless oder deinen eigenen Runpod-Pod.</x:v>
+      </x:c>
+      <x:c r="H1018" t="str">
+        <x:v>Added by v40.1.0 remote image providers</x:v>
+      </x:c>
+      <x:c r="I1018" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1018" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1019">
+      <x:c r="A1019" t="str">
+        <x:v>settings.image_provider_label</x:v>
+      </x:c>
+      <x:c r="B1019" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1019" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1019" t="str">
+        <x:v>Fournisseur d’images</x:v>
+      </x:c>
+      <x:c r="E1019" t="str">
+        <x:v>Image provider</x:v>
+      </x:c>
+      <x:c r="F1019" t="str">
+        <x:v>Proveedor de imágenes</x:v>
+      </x:c>
+      <x:c r="G1019" t="str">
+        <x:v>Bildanbieter</x:v>
+      </x:c>
+      <x:c r="H1019" t="str">
+        <x:v>Added by v40.1.0 remote image providers</x:v>
+      </x:c>
+      <x:c r="I1019" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1019" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1020">
+      <x:c r="A1020" t="str">
+        <x:v>settings.runpod_title</x:v>
+      </x:c>
+      <x:c r="B1020" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1020" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1020" t="str">
+        <x:v>Compte Runpod et arrêt automatique des Pods</x:v>
+      </x:c>
+      <x:c r="E1020" t="str">
+        <x:v>Runpod account and Pod policy</x:v>
+      </x:c>
+      <x:c r="F1020" t="str">
+        <x:v>Cuenta Runpod y política de Pods</x:v>
+      </x:c>
+      <x:c r="G1020" t="str">
+        <x:v>Runpod-Konto und Pod-Richtlinie</x:v>
+      </x:c>
+      <x:c r="H1020" t="str">
+        <x:v>Added by v40.1.0 Runpod controls</x:v>
+      </x:c>
+      <x:c r="I1020" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1020" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1021">
+      <x:c r="A1021" t="str">
+        <x:v>settings.runpod_hint</x:v>
+      </x:c>
+      <x:c r="B1021" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1021" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1021" t="str">
+        <x:v>AmiorAI ne vend ni calcul ni crédits. Cette clé pilote uniquement le compte Runpod qui t’appartient et qui te facture directement.</x:v>
+      </x:c>
+      <x:c r="E1021" t="str">
+        <x:v>AmiorAI never sells compute or credits. This key controls only the Runpod account owned and billed directly to you.</x:v>
+      </x:c>
+      <x:c r="F1021" t="str">
+        <x:v>AmiorAI no vende cómputo ni créditos. Esta clave controla únicamente tu propia cuenta de Runpod, facturada directamente por Runpod.</x:v>
+      </x:c>
+      <x:c r="G1021" t="str">
+        <x:v>AmiorAI verkauft weder Rechenleistung noch Guthaben. Dieser Schlüssel steuert ausschließlich dein eigenes, direkt von Runpod abgerechnetes Konto.</x:v>
+      </x:c>
+      <x:c r="H1021" t="str">
+        <x:v>Added by v40.1.0 Runpod controls</x:v>
+      </x:c>
+      <x:c r="I1021" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1021" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1022">
+      <x:c r="A1022" t="str">
+        <x:v>settings.llm_provider_lmstudio_opt</x:v>
+      </x:c>
+      <x:c r="B1022" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1022" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1022" t="str">
+        <x:v>LM Studio — local</x:v>
+      </x:c>
+      <x:c r="E1022" t="str">
+        <x:v>LM Studio — local</x:v>
+      </x:c>
+      <x:c r="F1022" t="str">
+        <x:v>LM Studio — local</x:v>
+      </x:c>
+      <x:c r="G1022" t="str">
+        <x:v>LM Studio — lokal</x:v>
+      </x:c>
+      <x:c r="H1022" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1022" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1022" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1023">
+      <x:c r="A1023" t="str">
+        <x:v>settings.llm_provider_openai_opt</x:v>
+      </x:c>
+      <x:c r="B1023" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1023" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1023" t="str">
+        <x:v>API compatible OpenAI — serveur de l’utilisateur</x:v>
+      </x:c>
+      <x:c r="E1023" t="str">
+        <x:v>OpenAI-compatible API — user-owned server</x:v>
+      </x:c>
+      <x:c r="F1023" t="str">
+        <x:v>API compatible con OpenAI — servidor del usuario</x:v>
+      </x:c>
+      <x:c r="G1023" t="str">
+        <x:v>OpenAI-kompatible API — eigener Server</x:v>
+      </x:c>
+      <x:c r="H1023" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1023" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1023" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1024">
+      <x:c r="A1024" t="str">
+        <x:v>settings.llm_provider_serverless_opt</x:v>
+      </x:c>
+      <x:c r="B1024" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1024" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1024" t="str">
+        <x:v>Runpod Serverless — vLLM</x:v>
+      </x:c>
+      <x:c r="E1024" t="str">
+        <x:v>Runpod Serverless — vLLM</x:v>
+      </x:c>
+      <x:c r="F1024" t="str">
+        <x:v>Runpod Serverless — vLLM</x:v>
+      </x:c>
+      <x:c r="G1024" t="str">
+        <x:v>Runpod Serverless — vLLM</x:v>
+      </x:c>
+      <x:c r="H1024" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1024" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1024" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1025">
+      <x:c r="A1025" t="str">
+        <x:v>settings.llm_provider_pod_opt</x:v>
+      </x:c>
+      <x:c r="B1025" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1025" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1025" t="str">
+        <x:v>Runpod Pod — vLLM</x:v>
+      </x:c>
+      <x:c r="E1025" t="str">
+        <x:v>Runpod Pod — vLLM</x:v>
+      </x:c>
+      <x:c r="F1025" t="str">
+        <x:v>Runpod Pod — vLLM</x:v>
+      </x:c>
+      <x:c r="G1025" t="str">
+        <x:v>Runpod Pod — vLLM</x:v>
+      </x:c>
+      <x:c r="H1025" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1025" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1025" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1026">
+      <x:c r="A1026" t="str">
+        <x:v>settings.llm_local_url_label</x:v>
+      </x:c>
+      <x:c r="B1026" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1026" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1026" t="str">
+        <x:v>Adresse du serveur LM Studio</x:v>
+      </x:c>
+      <x:c r="E1026" t="str">
+        <x:v>LM Studio server URL</x:v>
+      </x:c>
+      <x:c r="F1026" t="str">
+        <x:v>URL del servidor LM Studio</x:v>
+      </x:c>
+      <x:c r="G1026" t="str">
+        <x:v>Adresse des LM-Studio-Servers</x:v>
+      </x:c>
+      <x:c r="H1026" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1026" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1026" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1027">
+      <x:c r="A1027" t="str">
+        <x:v>settings.llm_conversation_model_label</x:v>
+      </x:c>
+      <x:c r="B1027" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1027" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1027" t="str">
+        <x:v>Modèle de conversation</x:v>
+      </x:c>
+      <x:c r="E1027" t="str">
+        <x:v>Conversation model</x:v>
+      </x:c>
+      <x:c r="F1027" t="str">
+        <x:v>Modelo de conversación</x:v>
+      </x:c>
+      <x:c r="G1027" t="str">
+        <x:v>Konversationsmodell</x:v>
+      </x:c>
+      <x:c r="H1027" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1027" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1027" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1028">
+      <x:c r="A1028" t="str">
+        <x:v>settings.llm_refresh_models_btn</x:v>
+      </x:c>
+      <x:c r="B1028" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1028" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1028" t="str">
+        <x:v>Actualiser la liste des modèles</x:v>
+      </x:c>
+      <x:c r="E1028" t="str">
+        <x:v>Refresh model list</x:v>
+      </x:c>
+      <x:c r="F1028" t="str">
+        <x:v>Actualizar lista de modelos</x:v>
+      </x:c>
+      <x:c r="G1028" t="str">
+        <x:v>Modellliste aktualisieren</x:v>
+      </x:c>
+      <x:c r="H1028" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1028" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1028" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1029">
+      <x:c r="A1029" t="str">
+        <x:v>settings.llm_local_start_hint</x:v>
+      </x:c>
+      <x:c r="B1029" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1029" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1029" t="str">
+        <x:v>Lance LM Studio, charge un modèle, démarre son serveur local, puis clique sur « Tester » ci-dessus.</x:v>
+      </x:c>
+      <x:c r="E1029" t="str">
+        <x:v>Start LM Studio, load a model, start its local server, then click Test above.</x:v>
+      </x:c>
+      <x:c r="F1029" t="str">
+        <x:v>Inicia LM Studio, carga un modelo, inicia su servidor local y pulsa Probar arriba.</x:v>
+      </x:c>
+      <x:c r="G1029" t="str">
+        <x:v>Starte LM Studio, lade ein Modell, starte den lokalen Server und klicke oben auf Testen.</x:v>
+      </x:c>
+      <x:c r="H1029" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1029" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1029" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1030">
+      <x:c r="A1030" t="str">
+        <x:v>settings.llm_remote_url_label</x:v>
+      </x:c>
+      <x:c r="B1030" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1030" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1030" t="str">
+        <x:v>Adresse de l’API compatible OpenAI</x:v>
+      </x:c>
+      <x:c r="E1030" t="str">
+        <x:v>OpenAI-compatible API URL</x:v>
+      </x:c>
+      <x:c r="F1030" t="str">
+        <x:v>URL de la API compatible con OpenAI</x:v>
+      </x:c>
+      <x:c r="G1030" t="str">
+        <x:v>Adresse der OpenAI-kompatiblen API</x:v>
+      </x:c>
+      <x:c r="H1030" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1030" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1030" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1031">
+      <x:c r="A1031" t="str">
+        <x:v>settings.llm_remote_model_label</x:v>
+      </x:c>
+      <x:c r="B1031" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1031" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1031" t="str">
+        <x:v>Identifiant du modèle de conversation</x:v>
+      </x:c>
+      <x:c r="E1031" t="str">
+        <x:v>Conversation model ID</x:v>
+      </x:c>
+      <x:c r="F1031" t="str">
+        <x:v>ID del modelo de conversación</x:v>
+      </x:c>
+      <x:c r="G1031" t="str">
+        <x:v>ID des Konversationsmodells</x:v>
+      </x:c>
+      <x:c r="H1031" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1031" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1031" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1032">
+      <x:c r="A1032" t="str">
+        <x:v>settings.remote_api_key_label</x:v>
+      </x:c>
+      <x:c r="B1032" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1032" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1032" t="str">
+        <x:v>Clé API du service (optionnelle)</x:v>
+      </x:c>
+      <x:c r="E1032" t="str">
+        <x:v>Service API key (optional)</x:v>
+      </x:c>
+      <x:c r="F1032" t="str">
+        <x:v>Clave API del servicio (opcional)</x:v>
+      </x:c>
+      <x:c r="G1032" t="str">
+        <x:v>API-Schlüssel des Dienstes (optional)</x:v>
+      </x:c>
+      <x:c r="H1032" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1032" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1032" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1033">
+      <x:c r="A1033" t="str">
+        <x:v>settings.secret_keep_placeholder</x:v>
+      </x:c>
+      <x:c r="B1033" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1033" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1033" t="str">
+        <x:v>Laisser vide pour conserver la clé enregistrée</x:v>
+      </x:c>
+      <x:c r="E1033" t="str">
+        <x:v>Leave blank to keep the saved key</x:v>
+      </x:c>
+      <x:c r="F1033" t="str">
+        <x:v>Déjalo vacío para conservar la clave guardada</x:v>
+      </x:c>
+      <x:c r="G1033" t="str">
+        <x:v>Leer lassen, um den gespeicherten Schlüssel zu behalten</x:v>
+      </x:c>
+      <x:c r="H1033" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1033" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1033" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1034">
+      <x:c r="A1034" t="str">
+        <x:v>settings.serverless_endpoint_label</x:v>
+      </x:c>
+      <x:c r="B1034" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1034" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1034" t="str">
+        <x:v>Identifiant de l’endpoint Runpod Serverless</x:v>
+      </x:c>
+      <x:c r="E1034" t="str">
+        <x:v>Runpod Serverless endpoint ID</x:v>
+      </x:c>
+      <x:c r="F1034" t="str">
+        <x:v>ID del endpoint Runpod Serverless</x:v>
+      </x:c>
+      <x:c r="G1034" t="str">
+        <x:v>ID des Runpod-Serverless-Endpunkts</x:v>
+      </x:c>
+      <x:c r="H1034" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1034" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1034" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1035">
+      <x:c r="A1035" t="str">
+        <x:v>settings.llm_serverless_model_label</x:v>
+      </x:c>
+      <x:c r="B1035" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1035" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1035" t="str">
+        <x:v>Identifiant du modèle exposé par vLLM</x:v>
+      </x:c>
+      <x:c r="E1035" t="str">
+        <x:v>Model ID exposed by vLLM</x:v>
+      </x:c>
+      <x:c r="F1035" t="str">
+        <x:v>ID del modelo expuesto por vLLM</x:v>
+      </x:c>
+      <x:c r="G1035" t="str">
+        <x:v>Von vLLM bereitgestellte Modell-ID</x:v>
+      </x:c>
+      <x:c r="H1035" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1035" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1035" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1036">
+      <x:c r="A1036" t="str">
+        <x:v>settings.llm_serverless_hint</x:v>
+      </x:c>
+      <x:c r="B1036" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1036" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1036" t="str">
+        <x:v>L’endpoint démarre un worker Flex à la demande. Réglage conseillé : 0 worker minimum et délai d’inactivité de 900 secondes.</x:v>
+      </x:c>
+      <x:c r="E1036" t="str">
+        <x:v>The endpoint starts a Flex worker on demand. Recommended setting: 0 minimum workers and a 900-second idle timeout.</x:v>
+      </x:c>
+      <x:c r="F1036" t="str">
+        <x:v>El endpoint inicia un worker Flex bajo demanda. Ajuste recomendado: 0 workers mínimos y 900 segundos de inactividad.</x:v>
+      </x:c>
+      <x:c r="G1036" t="str">
+        <x:v>Der Endpunkt startet bei Bedarf einen Flex-Worker. Empfohlen: 0 minimale Worker und 900 Sekunden Leerlaufzeit.</x:v>
+      </x:c>
+      <x:c r="H1036" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1036" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1036" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1037">
+      <x:c r="A1037" t="str">
+        <x:v>settings.runpod_pod_id_label</x:v>
+      </x:c>
+      <x:c r="B1037" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1037" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1037" t="str">
+        <x:v>Identifiant du Pod Runpod</x:v>
+      </x:c>
+      <x:c r="E1037" t="str">
+        <x:v>Runpod Pod ID</x:v>
+      </x:c>
+      <x:c r="F1037" t="str">
+        <x:v>ID del Pod Runpod</x:v>
+      </x:c>
+      <x:c r="G1037" t="str">
+        <x:v>Runpod-Pod-ID</x:v>
+      </x:c>
+      <x:c r="H1037" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1037" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1037" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1038">
+      <x:c r="A1038" t="str">
+        <x:v>settings.llm_pod_url_label</x:v>
+      </x:c>
+      <x:c r="B1038" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1038" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1038" t="str">
+        <x:v>Adresse API compatible OpenAI du Pod</x:v>
+      </x:c>
+      <x:c r="E1038" t="str">
+        <x:v>Pod OpenAI-compatible API URL</x:v>
+      </x:c>
+      <x:c r="F1038" t="str">
+        <x:v>URL de API compatible con OpenAI del Pod</x:v>
+      </x:c>
+      <x:c r="G1038" t="str">
+        <x:v>OpenAI-kompatible API-Adresse des Pods</x:v>
+      </x:c>
+      <x:c r="H1038" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1038" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1038" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1039">
+      <x:c r="A1039" t="str">
+        <x:v>settings.pod_start_timeout_label</x:v>
+      </x:c>
+      <x:c r="B1039" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1039" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1039" t="str">
+        <x:v>Attente maximale du démarrage du Pod (secondes)</x:v>
+      </x:c>
+      <x:c r="E1039" t="str">
+        <x:v>Maximum Pod startup wait (seconds)</x:v>
+      </x:c>
+      <x:c r="F1039" t="str">
+        <x:v>Espera máxima de inicio del Pod (segundos)</x:v>
+      </x:c>
+      <x:c r="G1039" t="str">
+        <x:v>Maximale Wartezeit beim Pod-Start (Sekunden)</x:v>
+      </x:c>
+      <x:c r="H1039" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1039" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1039" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1040">
+      <x:c r="A1040" t="str">
+        <x:v>settings.llm_pod_start_btn</x:v>
+      </x:c>
+      <x:c r="B1040" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1040" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1040" t="str">
+        <x:v>Démarrer le Pod LLM</x:v>
+      </x:c>
+      <x:c r="E1040" t="str">
+        <x:v>Start LLM Pod</x:v>
+      </x:c>
+      <x:c r="F1040" t="str">
+        <x:v>Iniciar Pod LLM</x:v>
+      </x:c>
+      <x:c r="G1040" t="str">
+        <x:v>LLM-Pod starten</x:v>
+      </x:c>
+      <x:c r="H1040" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1040" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1040" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1041">
+      <x:c r="A1041" t="str">
+        <x:v>settings.llm_pod_stop_btn</x:v>
+      </x:c>
+      <x:c r="B1041" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1041" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1041" t="str">
+        <x:v>Arrêter le Pod LLM</x:v>
+      </x:c>
+      <x:c r="E1041" t="str">
+        <x:v>Stop LLM Pod</x:v>
+      </x:c>
+      <x:c r="F1041" t="str">
+        <x:v>Detener Pod LLM</x:v>
+      </x:c>
+      <x:c r="G1041" t="str">
+        <x:v>LLM-Pod stoppen</x:v>
+      </x:c>
+      <x:c r="H1041" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1041" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1041" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1042">
+      <x:c r="A1042" t="str">
+        <x:v>settings.model_auto_placeholder</x:v>
+      </x:c>
+      <x:c r="B1042" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1042" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1042" t="str">
+        <x:v>— automatique / seul modèle chargé —</x:v>
+      </x:c>
+      <x:c r="E1042" t="str">
+        <x:v>— automatic / only loaded model —</x:v>
+      </x:c>
+      <x:c r="F1042" t="str">
+        <x:v>— automático / único modelo cargado —</x:v>
+      </x:c>
+      <x:c r="G1042" t="str">
+        <x:v>— automatisch / einzig geladenes Modell —</x:v>
+      </x:c>
+      <x:c r="H1042" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1042" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1042" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1043">
+      <x:c r="A1043" t="str">
+        <x:v>settings.model_detect_placeholder</x:v>
+      </x:c>
+      <x:c r="B1043" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1043" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1043" t="str">
+        <x:v>— détecter / choisir un modèle —</x:v>
+      </x:c>
+      <x:c r="E1043" t="str">
+        <x:v>— detect / select model —</x:v>
+      </x:c>
+      <x:c r="F1043" t="str">
+        <x:v>— detectar / elegir modelo —</x:v>
+      </x:c>
+      <x:c r="G1043" t="str">
+        <x:v>— Modell erkennen / auswählen —</x:v>
+      </x:c>
+      <x:c r="H1043" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1043" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1043" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1044">
+      <x:c r="A1044" t="str">
+        <x:v>settings.util_reuse_placeholder</x:v>
+      </x:c>
+      <x:c r="B1044" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1044" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1044" t="str">
+        <x:v>— réutiliser le modèle de conversation —</x:v>
+      </x:c>
+      <x:c r="E1044" t="str">
+        <x:v>— reuse conversation model —</x:v>
+      </x:c>
+      <x:c r="F1044" t="str">
+        <x:v>— reutilizar modelo de conversación —</x:v>
+      </x:c>
+      <x:c r="G1044" t="str">
+        <x:v>— Konversationsmodell wiederverwenden —</x:v>
+      </x:c>
+      <x:c r="H1044" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1044" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1044" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1045">
+      <x:c r="A1045" t="str">
+        <x:v>settings.image_provider_local_opt</x:v>
+      </x:c>
+      <x:c r="B1045" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1045" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1045" t="str">
+        <x:v>ComfyUI — local</x:v>
+      </x:c>
+      <x:c r="E1045" t="str">
+        <x:v>ComfyUI — local</x:v>
+      </x:c>
+      <x:c r="F1045" t="str">
+        <x:v>ComfyUI — local</x:v>
+      </x:c>
+      <x:c r="G1045" t="str">
+        <x:v>ComfyUI — lokal</x:v>
+      </x:c>
+      <x:c r="H1045" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1045" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1045" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1046">
+      <x:c r="A1046" t="str">
+        <x:v>settings.image_provider_remote_opt</x:v>
+      </x:c>
+      <x:c r="B1046" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1046" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1046" t="str">
+        <x:v>ComfyUI — API distante</x:v>
+      </x:c>
+      <x:c r="E1046" t="str">
+        <x:v>ComfyUI — remote API</x:v>
+      </x:c>
+      <x:c r="F1046" t="str">
+        <x:v>ComfyUI — API remota</x:v>
+      </x:c>
+      <x:c r="G1046" t="str">
+        <x:v>ComfyUI — Remote-API</x:v>
+      </x:c>
+      <x:c r="H1046" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1046" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1046" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1047">
+      <x:c r="A1047" t="str">
+        <x:v>settings.image_provider_serverless_opt</x:v>
+      </x:c>
+      <x:c r="B1047" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1047" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1047" t="str">
+        <x:v>Runpod Serverless — worker ComfyUI</x:v>
+      </x:c>
+      <x:c r="E1047" t="str">
+        <x:v>Runpod Serverless — ComfyUI worker</x:v>
+      </x:c>
+      <x:c r="F1047" t="str">
+        <x:v>Runpod Serverless — worker ComfyUI</x:v>
+      </x:c>
+      <x:c r="G1047" t="str">
+        <x:v>Runpod Serverless — ComfyUI-Worker</x:v>
+      </x:c>
+      <x:c r="H1047" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1047" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1047" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1048">
+      <x:c r="A1048" t="str">
+        <x:v>settings.image_provider_pod_opt</x:v>
+      </x:c>
+      <x:c r="B1048" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1048" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1048" t="str">
+        <x:v>Runpod Pod — ComfyUI</x:v>
+      </x:c>
+      <x:c r="E1048" t="str">
+        <x:v>Runpod Pod — ComfyUI</x:v>
+      </x:c>
+      <x:c r="F1048" t="str">
+        <x:v>Runpod Pod — ComfyUI</x:v>
+      </x:c>
+      <x:c r="G1048" t="str">
+        <x:v>Runpod Pod — ComfyUI</x:v>
+      </x:c>
+      <x:c r="H1048" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1048" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1048" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1049">
+      <x:c r="A1049" t="str">
+        <x:v>settings.image_remote_url_label</x:v>
+      </x:c>
+      <x:c r="B1049" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1049" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1049" t="str">
+        <x:v>Adresse de l’API ComfyUI distante</x:v>
+      </x:c>
+      <x:c r="E1049" t="str">
+        <x:v>Remote ComfyUI API URL</x:v>
+      </x:c>
+      <x:c r="F1049" t="str">
+        <x:v>URL de la API ComfyUI remota</x:v>
+      </x:c>
+      <x:c r="G1049" t="str">
+        <x:v>Adresse der entfernten ComfyUI-API</x:v>
+      </x:c>
+      <x:c r="H1049" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1049" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1049" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1050">
+      <x:c r="A1050" t="str">
+        <x:v>settings.image_serverless_hint</x:v>
+      </x:c>
+      <x:c r="B1050" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1050" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1050" t="str">
+        <x:v>Utilise le format AmiorAI pour ComfyUI : workflow et images de référence facultatives. L’endpoint démarre à la première génération.</x:v>
+      </x:c>
+      <x:c r="E1050" t="str">
+        <x:v>Uses the AmiorAI ComfyUI format: workflow plus optional reference images. The endpoint starts on the first generation.</x:v>
+      </x:c>
+      <x:c r="F1050" t="str">
+        <x:v>Usa el formato ComfyUI de AmiorAI: workflow e imágenes de referencia opcionales. El endpoint se inicia en la primera generación.</x:v>
+      </x:c>
+      <x:c r="G1050" t="str">
+        <x:v>Verwendet das AmiorAI-ComfyUI-Format: Workflow plus optionale Referenzbilder. Der Endpunkt startet bei der ersten Generierung.</x:v>
+      </x:c>
+      <x:c r="H1050" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1050" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1050" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1051">
+      <x:c r="A1051" t="str">
+        <x:v>settings.image_pod_url_label</x:v>
+      </x:c>
+      <x:c r="B1051" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1051" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1051" t="str">
+        <x:v>Adresse API ComfyUI du Pod</x:v>
+      </x:c>
+      <x:c r="E1051" t="str">
+        <x:v>Pod ComfyUI API URL</x:v>
+      </x:c>
+      <x:c r="F1051" t="str">
+        <x:v>URL de API ComfyUI del Pod</x:v>
+      </x:c>
+      <x:c r="G1051" t="str">
+        <x:v>ComfyUI-API-Adresse des Pods</x:v>
+      </x:c>
+      <x:c r="H1051" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1051" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1051" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1052">
+      <x:c r="A1052" t="str">
+        <x:v>settings.image_pod_start_btn</x:v>
+      </x:c>
+      <x:c r="B1052" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1052" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1052" t="str">
+        <x:v>Démarrer le Pod image</x:v>
+      </x:c>
+      <x:c r="E1052" t="str">
+        <x:v>Start Image Pod</x:v>
+      </x:c>
+      <x:c r="F1052" t="str">
+        <x:v>Iniciar Pod de imagen</x:v>
+      </x:c>
+      <x:c r="G1052" t="str">
+        <x:v>Bild-Pod starten</x:v>
+      </x:c>
+      <x:c r="H1052" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1052" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1052" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1053">
+      <x:c r="A1053" t="str">
+        <x:v>settings.image_pod_stop_btn</x:v>
+      </x:c>
+      <x:c r="B1053" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1053" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1053" t="str">
+        <x:v>Arrêter le Pod image</x:v>
+      </x:c>
+      <x:c r="E1053" t="str">
+        <x:v>Stop Image Pod</x:v>
+      </x:c>
+      <x:c r="F1053" t="str">
+        <x:v>Detener Pod de imagen</x:v>
+      </x:c>
+      <x:c r="G1053" t="str">
+        <x:v>Bild-Pod stoppen</x:v>
+      </x:c>
+      <x:c r="H1053" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1053" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1053" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1054">
+      <x:c r="A1054" t="str">
+        <x:v>settings.image_resolution_hint</x:v>
+      </x:c>
+      <x:c r="B1054" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1054" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1054" t="str">
+        <x:v>S’applique à toutes les générations sauf aux aperçus (512×512 fixe). Duo, Trio et Groupe utilisent la résolution de leur propre workflow.</x:v>
+      </x:c>
+      <x:c r="E1054" t="str">
+        <x:v>Applies to all generations except previews (fixed 512×512). Duo, Trio, and Group use their own workflow resolution.</x:v>
+      </x:c>
+      <x:c r="F1054" t="str">
+        <x:v>Se aplica a todas las generaciones excepto las vistas previas (512×512 fijo). Dúo, Trío y Grupo usan la resolución de su propio workflow.</x:v>
+      </x:c>
+      <x:c r="G1054" t="str">
+        <x:v>Gilt für alle Generierungen außer Vorschauen (fest 512×512). Duo, Trio und Gruppe verwenden die Auflösung ihres eigenen Workflows.</x:v>
+      </x:c>
+      <x:c r="H1054" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1054" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1054" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1055">
+      <x:c r="A1055" t="str">
+        <x:v>settings.runpod_api_key_label</x:v>
+      </x:c>
+      <x:c r="B1055" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1055" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1055" t="str">
+        <x:v>Clé API Runpod</x:v>
+      </x:c>
+      <x:c r="E1055" t="str">
+        <x:v>Runpod API key</x:v>
+      </x:c>
+      <x:c r="F1055" t="str">
+        <x:v>Clave API de Runpod</x:v>
+      </x:c>
+      <x:c r="G1055" t="str">
+        <x:v>Runpod-API-Schlüssel</x:v>
+      </x:c>
+      <x:c r="H1055" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1055" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1055" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1056">
+      <x:c r="A1056" t="str">
+        <x:v>settings.runpod_auto_stop_label</x:v>
+      </x:c>
+      <x:c r="B1056" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1056" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1056" t="str">
+        <x:v>Arrêter automatiquement un Pod après une période d’inactivité</x:v>
+      </x:c>
+      <x:c r="E1056" t="str">
+        <x:v>Automatically stop a Pod after inactivity</x:v>
+      </x:c>
+      <x:c r="F1056" t="str">
+        <x:v>Detener automáticamente un Pod tras un periodo de inactividad</x:v>
+      </x:c>
+      <x:c r="G1056" t="str">
+        <x:v>Pod nach Inaktivität automatisch stoppen</x:v>
+      </x:c>
+      <x:c r="H1056" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1056" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1056" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1057">
+      <x:c r="A1057" t="str">
+        <x:v>settings.runpod_idle_label</x:v>
+      </x:c>
+      <x:c r="B1057" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1057" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1057" t="str">
+        <x:v>Délai d’inactivité (minutes)</x:v>
+      </x:c>
+      <x:c r="E1057" t="str">
+        <x:v>Inactivity delay (minutes)</x:v>
+      </x:c>
+      <x:c r="F1057" t="str">
+        <x:v>Tiempo de inactividad (minutos)</x:v>
+      </x:c>
+      <x:c r="G1057" t="str">
+        <x:v>Inaktivitätsdauer (Minuten)</x:v>
+      </x:c>
+      <x:c r="H1057" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1057" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1057" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1058">
+      <x:c r="A1058" t="str">
+        <x:v>settings.runpod_auto_stop_hint</x:v>
+      </x:c>
+      <x:c r="B1058" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1058" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1058" t="str">
+        <x:v>Le compte à rebours commence après la dernière requête terminée. Une génération de texte ou d’image, un envoi ou un téléchargement en cours empêche l’arrêt. Un crash ou une coupure ne permet pas de garantir la commande d’arrêt : vérifie le tableau de bord Runpod.</x:v>
+      </x:c>
+      <x:c r="E1058" t="str">
+        <x:v>The countdown starts after the last completed request. Active text or image generation, upload, or download prevents automatic stop. A crash or power loss cannot guarantee the stop command; verify the Runpod dashboard.</x:v>
+      </x:c>
+      <x:c r="F1058" t="str">
+        <x:v>La cuenta atrás empieza tras la última solicitud terminada. Una generación de texto o imagen, una subida o una descarga activa evita la detención. Un fallo o corte eléctrico no garantiza la orden de parada; comprueba el panel de Runpod.</x:v>
+      </x:c>
+      <x:c r="G1058" t="str">
+        <x:v>Der Countdown beginnt nach der letzten abgeschlossenen Anfrage. Laufende Text- oder Bildgenerierung sowie Uploads oder Downloads verhindern den Stopp. Bei Absturz oder Stromausfall kann der Stoppbefehl nicht garantiert werden; prüfe das Runpod-Dashboard.</x:v>
+      </x:c>
+      <x:c r="H1058" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1058" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1058" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1059">
+      <x:c r="A1059" t="str">
+        <x:v>settings.models_reading</x:v>
+      </x:c>
+      <x:c r="B1059" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1059" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1059" t="str">
+        <x:v>Lecture des modèles depuis {provider}…</x:v>
+      </x:c>
+      <x:c r="E1059" t="str">
+        <x:v>Reading models from {provider}…</x:v>
+      </x:c>
+      <x:c r="F1059" t="str">
+        <x:v>Leyendo modelos desde {provider}…</x:v>
+      </x:c>
+      <x:c r="G1059" t="str">
+        <x:v>Modelle werden von {provider} gelesen…</x:v>
+      </x:c>
+      <x:c r="H1059" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1059" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1059" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1060">
+      <x:c r="A1060" t="str">
+        <x:v>settings.models_exposed</x:v>
+      </x:c>
+      <x:c r="B1060" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1060" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1060" t="str">
+        <x:v>{count} modèle(s) exposé(s) par {provider}.</x:v>
+      </x:c>
+      <x:c r="E1060" t="str">
+        <x:v>{count} model(s) exposed by {provider}.</x:v>
+      </x:c>
+      <x:c r="F1060" t="str">
+        <x:v>{count} modelo(s) expuesto(s) por {provider}.</x:v>
+      </x:c>
+      <x:c r="G1060" t="str">
+        <x:v>{count} Modell(e) von {provider} bereitgestellt.</x:v>
+      </x:c>
+      <x:c r="H1060" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1060" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1060" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1061">
+      <x:c r="A1061" t="str">
+        <x:v>settings.provider_unavailable</x:v>
+      </x:c>
+      <x:c r="B1061" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1061" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1061" t="str">
+        <x:v>{provider} est indisponible.</x:v>
+      </x:c>
+      <x:c r="E1061" t="str">
+        <x:v>{provider} is unavailable.</x:v>
+      </x:c>
+      <x:c r="F1061" t="str">
+        <x:v>{provider} no está disponible.</x:v>
+      </x:c>
+      <x:c r="G1061" t="str">
+        <x:v>{provider} ist nicht verfügbar.</x:v>
+      </x:c>
+      <x:c r="H1061" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1061" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1061" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1062">
+      <x:c r="A1062" t="str">
+        <x:v>settings.model_not_exposed</x:v>
+      </x:c>
+      <x:c r="B1062" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1062" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1062" t="str">
+        <x:v>{model} (non exposé actuellement)</x:v>
+      </x:c>
+      <x:c r="E1062" t="str">
+        <x:v>{model} (not currently exposed)</x:v>
+      </x:c>
+      <x:c r="F1062" t="str">
+        <x:v>{model} (no expuesto actualmente)</x:v>
+      </x:c>
+      <x:c r="G1062" t="str">
+        <x:v>{model} (derzeit nicht bereitgestellt)</x:v>
+      </x:c>
+      <x:c r="H1062" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1062" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1062" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1063">
+      <x:c r="A1063" t="str">
+        <x:v>settings.key_saved</x:v>
+      </x:c>
+      <x:c r="B1063" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1063" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1063" t="str">
+        <x:v>✓ {label} enregistrée dans {storage}</x:v>
+      </x:c>
+      <x:c r="E1063" t="str">
+        <x:v>✓ {label} saved in {storage}</x:v>
+      </x:c>
+      <x:c r="F1063" t="str">
+        <x:v>✓ {label} guardada en {storage}</x:v>
+      </x:c>
+      <x:c r="G1063" t="str">
+        <x:v>✓ {label} in {storage} gespeichert</x:v>
+      </x:c>
+      <x:c r="H1063" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1063" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1063" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1064">
+      <x:c r="A1064" t="str">
+        <x:v>settings.key_not_configured</x:v>
+      </x:c>
+      <x:c r="B1064" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1064" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1064" t="str">
+        <x:v>{label} non configurée.</x:v>
+      </x:c>
+      <x:c r="E1064" t="str">
+        <x:v>{label} not configured.</x:v>
+      </x:c>
+      <x:c r="F1064" t="str">
+        <x:v>{label} no configurada.</x:v>
+      </x:c>
+      <x:c r="G1064" t="str">
+        <x:v>{label} nicht konfiguriert.</x:v>
+      </x:c>
+      <x:c r="H1064" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1064" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1064" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1065">
+      <x:c r="A1065" t="str">
+        <x:v>settings.key_runpod_label</x:v>
+      </x:c>
+      <x:c r="B1065" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1065" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1065" t="str">
+        <x:v>Clé du compte Runpod</x:v>
+      </x:c>
+      <x:c r="E1065" t="str">
+        <x:v>Runpod account key</x:v>
+      </x:c>
+      <x:c r="F1065" t="str">
+        <x:v>Clave de la cuenta Runpod</x:v>
+      </x:c>
+      <x:c r="G1065" t="str">
+        <x:v>Runpod-Kontoschlüssel</x:v>
+      </x:c>
+      <x:c r="H1065" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1065" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1065" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1066">
+      <x:c r="A1066" t="str">
+        <x:v>settings.key_llm_label</x:v>
+      </x:c>
+      <x:c r="B1066" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1066" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1066" t="str">
+        <x:v>Clé du service LLM</x:v>
+      </x:c>
+      <x:c r="E1066" t="str">
+        <x:v>LLM service key</x:v>
+      </x:c>
+      <x:c r="F1066" t="str">
+        <x:v>Clave del servicio LLM</x:v>
+      </x:c>
+      <x:c r="G1066" t="str">
+        <x:v>LLM-Dienstschlüssel</x:v>
+      </x:c>
+      <x:c r="H1066" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1066" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1066" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1067">
+      <x:c r="A1067" t="str">
+        <x:v>settings.key_image_label</x:v>
+      </x:c>
+      <x:c r="B1067" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1067" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1067" t="str">
+        <x:v>Clé du service d’image</x:v>
+      </x:c>
+      <x:c r="E1067" t="str">
+        <x:v>Image service key</x:v>
+      </x:c>
+      <x:c r="F1067" t="str">
+        <x:v>Clave del servicio de imagen</x:v>
+      </x:c>
+      <x:c r="G1067" t="str">
+        <x:v>Bilddienstschlüssel</x:v>
+      </x:c>
+      <x:c r="H1067" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1067" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1067" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1068">
+      <x:c r="A1068" t="str">
+        <x:v>settings.secure_storage</x:v>
+      </x:c>
+      <x:c r="B1068" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1068" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1068" t="str">
+        <x:v>le stockage sécurisé</x:v>
+      </x:c>
+      <x:c r="E1068" t="str">
+        <x:v>secure storage</x:v>
+      </x:c>
+      <x:c r="F1068" t="str">
+        <x:v>almacenamiento seguro</x:v>
+      </x:c>
+      <x:c r="G1068" t="str">
+        <x:v>sicherem Speicher</x:v>
+      </x:c>
+      <x:c r="H1068" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1068" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1068" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1069">
+      <x:c r="A1069" t="str">
+        <x:v>settings.checking_provider</x:v>
+      </x:c>
+      <x:c r="B1069" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1069" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1069" t="str">
+        <x:v>Vérification de {provider}…</x:v>
+      </x:c>
+      <x:c r="E1069" t="str">
+        <x:v>Checking {provider}…</x:v>
+      </x:c>
+      <x:c r="F1069" t="str">
+        <x:v>Comprobando {provider}…</x:v>
+      </x:c>
+      <x:c r="G1069" t="str">
+        <x:v>{provider} wird geprüft…</x:v>
+      </x:c>
+      <x:c r="H1069" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1069" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1069" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1070">
+      <x:c r="A1070" t="str">
+        <x:v>settings.provider_connected</x:v>
+      </x:c>
+      <x:c r="B1070" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1070" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1070" t="str">
+        <x:v>✓ {provider} connecté</x:v>
+      </x:c>
+      <x:c r="E1070" t="str">
+        <x:v>✓ {provider} connected</x:v>
+      </x:c>
+      <x:c r="F1070" t="str">
+        <x:v>✓ {provider} conectado</x:v>
+      </x:c>
+      <x:c r="G1070" t="str">
+        <x:v>✓ {provider} verbunden</x:v>
+      </x:c>
+      <x:c r="H1070" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1070" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1070" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1071">
+      <x:c r="A1071" t="str">
+        <x:v>settings.provider_unreachable</x:v>
+      </x:c>
+      <x:c r="B1071" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1071" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1071" t="str">
+        <x:v>{provider} inaccessible</x:v>
+      </x:c>
+      <x:c r="E1071" t="str">
+        <x:v>{provider} unreachable</x:v>
+      </x:c>
+      <x:c r="F1071" t="str">
+        <x:v>{provider} inaccesible</x:v>
+      </x:c>
+      <x:c r="G1071" t="str">
+        <x:v>{provider} nicht erreichbar</x:v>
+      </x:c>
+      <x:c r="H1071" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1071" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1071" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1072">
+      <x:c r="A1072" t="str">
+        <x:v>settings.available_model_ids</x:v>
+      </x:c>
+      <x:c r="B1072" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1072" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1072" t="str">
+        <x:v>Identifiants disponibles : {models}</x:v>
+      </x:c>
+      <x:c r="E1072" t="str">
+        <x:v>Available model IDs: {models}</x:v>
+      </x:c>
+      <x:c r="F1072" t="str">
+        <x:v>IDs de modelo disponibles: {models}</x:v>
+      </x:c>
+      <x:c r="G1072" t="str">
+        <x:v>Verfügbare Modell-IDs: {models}</x:v>
+      </x:c>
+      <x:c r="H1072" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1072" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1072" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1073">
+      <x:c r="A1073" t="str">
+        <x:v>settings.pod_unknown</x:v>
+      </x:c>
+      <x:c r="B1073" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1073" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1073" t="str">
+        <x:v>état inconnu</x:v>
+      </x:c>
+      <x:c r="E1073" t="str">
+        <x:v>unknown status</x:v>
+      </x:c>
+      <x:c r="F1073" t="str">
+        <x:v>estado desconocido</x:v>
+      </x:c>
+      <x:c r="G1073" t="str">
+        <x:v>unbekannter Status</x:v>
+      </x:c>
+      <x:c r="H1073" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1073" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1073" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1074">
+      <x:c r="A1074" t="str">
+        <x:v>settings.pod_not_configured</x:v>
+      </x:c>
+      <x:c r="B1074" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1074" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1074" t="str">
+        <x:v>non configuré</x:v>
+      </x:c>
+      <x:c r="E1074" t="str">
+        <x:v>not configured</x:v>
+      </x:c>
+      <x:c r="F1074" t="str">
+        <x:v>no configurado</x:v>
+      </x:c>
+      <x:c r="G1074" t="str">
+        <x:v>nicht konfiguriert</x:v>
+      </x:c>
+      <x:c r="H1074" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1074" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1074" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1075">
+      <x:c r="A1075" t="str">
+        <x:v>settings.pod_auto_stop_in</x:v>
+      </x:c>
+      <x:c r="B1075" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1075" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1075" t="str">
+        <x:v>{status} · arrêt automatique dans {minutes} min</x:v>
+      </x:c>
+      <x:c r="E1075" t="str">
+        <x:v>{status} · auto-stop in {minutes} min</x:v>
+      </x:c>
+      <x:c r="F1075" t="str">
+        <x:v>{status} · parada automática en {minutes} min</x:v>
+      </x:c>
+      <x:c r="G1075" t="str">
+        <x:v>{status} · automatischer Stopp in {minutes} Min.</x:v>
+      </x:c>
+      <x:c r="H1075" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1075" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1075" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1076">
+      <x:c r="A1076" t="str">
+        <x:v>settings.pod_action_start</x:v>
+      </x:c>
+      <x:c r="B1076" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1076" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1076" t="str">
+        <x:v>démarrage</x:v>
+      </x:c>
+      <x:c r="E1076" t="str">
+        <x:v>starting</x:v>
+      </x:c>
+      <x:c r="F1076" t="str">
+        <x:v>iniciando</x:v>
+      </x:c>
+      <x:c r="G1076" t="str">
+        <x:v>Start läuft</x:v>
+      </x:c>
+      <x:c r="H1076" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1076" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1076" t="str">
+        <x:v>ok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1077">
+      <x:c r="A1077" t="str">
+        <x:v>settings.pod_action_stop</x:v>
+      </x:c>
+      <x:c r="B1077" t="str">
+        <x:v>settings</x:v>
+      </x:c>
+      <x:c r="C1077" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="D1077" t="str">
+        <x:v>arrêt</x:v>
+      </x:c>
+      <x:c r="E1077" t="str">
+        <x:v>stopping</x:v>
+      </x:c>
+      <x:c r="F1077" t="str">
+        <x:v>deteniendo</x:v>
+      </x:c>
+      <x:c r="G1077" t="str">
+        <x:v>Stopp läuft</x:v>
+      </x:c>
+      <x:c r="H1077" t="str">
+        <x:v>Added by v40.1.0 remote providers UI</x:v>
+      </x:c>
+      <x:c r="I1077" t="str">
+        <x:v>resources/i18n/locales/*.json</x:v>
+      </x:c>
+      <x:c r="J1077" t="str">
         <x:v>ok</x:v>
       </x:c>
     </x:row>
@@ -32281,7 +34273,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>40.0.9</x:v>
+        <x:v>40.1.0</x:v>
       </x:c>
     </x:row>
     <x:row r="6">

</xml_diff>